<commit_message>
fix(events): souhrn kategorií se tiskne na stránce se soupisem výdajů
Soupis výdajů je na výšku a sloupce se souhrnem kategorií (H, I) se na stránku
nevešly, takže se tiskly samy na další list. Šablona si o zúžení na jednu stránku
říkala už dřív, ale s pageSetUpPr/@fitToPage="false" se na to nehledělo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q5cKia4F6Pmsk3Kc4emVSZ
</commit_message>
<xml_diff>
--- a/backend/assets/uctovani-v7.xlsx
+++ b/backend/assets/uctovani-v7.xlsx
@@ -10360,7 +10360,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -11057,7 +11057,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
revert(events): tisková oblast soupisu výdajů zpět beze změny
Zúžení listu na jednu stránku na šířku vracím zpátky — souhrn kategorií se tedy
zase tiskne na vlastní list, tak jak to bylo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q5cKia4F6Pmsk3Kc4emVSZ
</commit_message>
<xml_diff>
--- a/backend/assets/uctovani-v7.xlsx
+++ b/backend/assets/uctovani-v7.xlsx
@@ -10360,7 +10360,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="true"/>
+    <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -11057,7 +11057,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
fix(events): souhrn kategorií zpět na stránku se soupisem výdajů
Vrací zúžení listu na jednu stránku na šířku. Bez něj sloupce se souhrnem (H, I)
u soupisu na výšku přetečou a vytisknou se samy na další list.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q5cKia4F6Pmsk3Kc4emVSZ
</commit_message>
<xml_diff>
--- a/backend/assets/uctovani-v7.xlsx
+++ b/backend/assets/uctovani-v7.xlsx
@@ -10360,7 +10360,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -11057,7 +11057,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>